<commit_message>
20230619-2225 Get 20230611 dividend data.
</commit_message>
<xml_diff>
--- a/Data/EXCEL/Transfer/dividend/20230611/0050-dividend-20230611.xlsx
+++ b/Data/EXCEL/Transfer/dividend/20230611/0050-dividend-20230611.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspaces\xls2xlsx\20230611\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspaces\xls2xlsx\20230611\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A60B763C-8337-46A5-ABFB-A15516BCE1FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D5081682-0E82-4F44-8E1E-72DB3F18551D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="555" yWindow="1245" windowWidth="25395" windowHeight="18240"/>
   </bookViews>

</xml_diff>